<commit_message>
TMTT0048687_JobTypes Final Changes Aug 28 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTT0047192_VerifyNewFieldCompetitiveAddedToCMNewOpportunityEngagementCounterpartyPage.xlsx
+++ b/TestData/LV_TMTT0047192_VerifyNewFieldCompetitiveAddedToCMNewOpportunityEngagementCounterpartyPage.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B475501A-67C0-4EE5-8EF1-270AFAF681AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D33C4F5-CDB1-4DA8-BC96-77F75DBD18B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="548" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="101">
   <si>
     <t>James Craven</t>
   </si>
@@ -323,9 +323,6 @@
     <t>Printable View</t>
   </si>
   <si>
-    <t>Engagement_Competitive</t>
-  </si>
-  <si>
     <t>EngagementsName</t>
   </si>
   <si>
@@ -338,10 +335,19 @@
     <t>OpportunityNo</t>
   </si>
   <si>
-    <t>Opportunity_Competitive</t>
-  </si>
-  <si>
-    <t>145024</t>
+    <t>145511</t>
+  </si>
+  <si>
+    <t>Buyside</t>
+  </si>
+  <si>
+    <t>144822</t>
+  </si>
+  <si>
+    <t>Competitive_Engagement</t>
+  </si>
+  <si>
+    <t>Competitive_Opportunity</t>
   </si>
 </sst>
 </file>
@@ -719,13 +725,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -733,10 +739,10 @@
         <v>98</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1211,24 +1217,24 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" t="s">
         <v>97</v>
-      </c>
-      <c r="C2" t="s">
-        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>